<commit_message>
Feb 1 2024 T1432changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25EAC2AC-9332-411B-BC7D-4A5F94260813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789B0483-6441-4820-9215-423A1F0C39A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -2543,7 +2543,7 @@
     <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
@@ -2557,35 +2557,38 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>93</v>
+      <c r="D2" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>100</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" t="s">
         <v>43</v>
       </c>
+      <c r="D3" s="6" t="s">
+        <v>84</v>
+      </c>
       <c r="E3">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2598,11 +2601,11 @@
       <c r="C4" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>76</v>
+      <c r="D4" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2616,10 +2619,10 @@
         <v>43</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2633,10 +2636,10 @@
         <v>43</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2650,10 +2653,10 @@
         <v>43</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2667,10 +2670,10 @@
         <v>43</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2684,13 +2687,13 @@
         <v>43</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>100</v>
       </c>
@@ -2700,11 +2703,11 @@
       <c r="C10" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>89</v>
+      <c r="D10" s="7" t="s">
+        <v>91</v>
       </c>
       <c r="E10">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2717,45 +2720,42 @@
       <c r="C11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>90</v>
+      <c r="D11" s="8" t="s">
+        <v>92</v>
       </c>
       <c r="E11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>91</v>
+      <c r="D12" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="E12">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>100</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="E13">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apr 16 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE4D515-F067-41F6-A45E-4D490A8D6695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B80AA7-E63F-4277-90B1-5BE1C0EFE54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="163">
   <si>
     <t>James Craven</t>
   </si>
@@ -241,9 +241,6 @@
   </si>
   <si>
     <t>Kristian M. Whalen</t>
-  </si>
-  <si>
-    <t>William Peluchiwski</t>
   </si>
   <si>
     <t>Eric Cartier</t>
@@ -972,12 +969,12 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1002,17 +999,17 @@
         <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1031,26 +1028,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1063,7 +1060,7 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1075,26 +1072,26 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1145,7 +1142,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1166,7 +1163,7 @@
     <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -1255,7 +1252,7 @@
         <v>34</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>35</v>
@@ -1264,7 +1261,7 @@
         <v>36</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>37</v>
@@ -1278,10 +1275,10 @@
         <v>38</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E2" t="s">
         <v>39</v>
@@ -1302,7 +1299,7 @@
         <v>40</v>
       </c>
       <c r="K2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L2" t="s">
         <v>42</v>
@@ -1311,7 +1308,7 @@
         <v>43</v>
       </c>
       <c r="N2" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>44</v>
@@ -1344,19 +1341,19 @@
         <v>50</v>
       </c>
       <c r="Y2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z2" t="s">
         <v>51</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD2" t="s">
         <v>52</v>
@@ -1373,10 +1370,10 @@
         <v>38</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E3" t="s">
         <v>39</v>
@@ -1397,7 +1394,7 @@
         <v>40</v>
       </c>
       <c r="K3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L3" t="s">
         <v>42</v>
@@ -1406,7 +1403,7 @@
         <v>43</v>
       </c>
       <c r="N3" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>44</v>
@@ -1439,19 +1436,19 @@
         <v>50</v>
       </c>
       <c r="Y3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z3" t="s">
         <v>51</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB3" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD3" t="s">
         <v>40</v>
@@ -1468,10 +1465,10 @@
         <v>38</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E4" t="s">
         <v>39</v>
@@ -1492,7 +1489,7 @@
         <v>40</v>
       </c>
       <c r="K4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L4" t="s">
         <v>42</v>
@@ -1501,7 +1498,7 @@
         <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>44</v>
@@ -1534,19 +1531,19 @@
         <v>50</v>
       </c>
       <c r="Y4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z4" t="s">
         <v>51</v>
       </c>
       <c r="AA4" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB4" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD4" t="s">
         <v>52</v>
@@ -1563,10 +1560,10 @@
         <v>38</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E5" t="s">
         <v>39</v>
@@ -1587,7 +1584,7 @@
         <v>40</v>
       </c>
       <c r="K5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L5" t="s">
         <v>42</v>
@@ -1596,7 +1593,7 @@
         <v>43</v>
       </c>
       <c r="N5" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>44</v>
@@ -1629,19 +1626,19 @@
         <v>50</v>
       </c>
       <c r="Y5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z5" t="s">
         <v>51</v>
       </c>
       <c r="AA5" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD5" t="s">
         <v>40</v>
@@ -1658,10 +1655,10 @@
         <v>38</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E6" t="s">
         <v>39</v>
@@ -1682,7 +1679,7 @@
         <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L6" t="s">
         <v>42</v>
@@ -1691,7 +1688,7 @@
         <v>43</v>
       </c>
       <c r="N6" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>44</v>
@@ -1724,19 +1721,19 @@
         <v>50</v>
       </c>
       <c r="Y6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z6" t="s">
         <v>51</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD6" t="s">
         <v>52</v>
@@ -1753,10 +1750,10 @@
         <v>38</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E7" t="s">
         <v>39</v>
@@ -1777,7 +1774,7 @@
         <v>40</v>
       </c>
       <c r="K7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L7" t="s">
         <v>42</v>
@@ -1786,7 +1783,7 @@
         <v>43</v>
       </c>
       <c r="N7" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>44</v>
@@ -1819,19 +1816,19 @@
         <v>50</v>
       </c>
       <c r="Y7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z7" t="s">
         <v>51</v>
       </c>
       <c r="AA7" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD7" t="s">
         <v>40</v>
@@ -1848,10 +1845,10 @@
         <v>38</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E8" t="s">
         <v>39</v>
@@ -1872,7 +1869,7 @@
         <v>40</v>
       </c>
       <c r="K8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L8" t="s">
         <v>42</v>
@@ -1881,7 +1878,7 @@
         <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>44</v>
@@ -1914,19 +1911,19 @@
         <v>50</v>
       </c>
       <c r="Y8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z8" t="s">
         <v>51</v>
       </c>
       <c r="AA8" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB8" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD8" t="s">
         <v>52</v>
@@ -1943,10 +1940,10 @@
         <v>38</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E9" t="s">
         <v>39</v>
@@ -1967,7 +1964,7 @@
         <v>40</v>
       </c>
       <c r="K9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L9" t="s">
         <v>42</v>
@@ -1976,7 +1973,7 @@
         <v>43</v>
       </c>
       <c r="N9" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>44</v>
@@ -2009,19 +2006,19 @@
         <v>50</v>
       </c>
       <c r="Y9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z9" t="s">
         <v>51</v>
       </c>
       <c r="AA9" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD9" t="s">
         <v>40</v>
@@ -2038,10 +2035,10 @@
         <v>38</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E10" t="s">
         <v>39</v>
@@ -2062,7 +2059,7 @@
         <v>40</v>
       </c>
       <c r="K10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L10" t="s">
         <v>42</v>
@@ -2071,7 +2068,7 @@
         <v>43</v>
       </c>
       <c r="N10" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>44</v>
@@ -2104,19 +2101,19 @@
         <v>50</v>
       </c>
       <c r="Y10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z10" t="s">
         <v>51</v>
       </c>
       <c r="AA10" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB10" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD10" t="s">
         <v>52</v>
@@ -2133,10 +2130,10 @@
         <v>38</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E11" t="s">
         <v>39</v>
@@ -2157,7 +2154,7 @@
         <v>40</v>
       </c>
       <c r="K11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L11" t="s">
         <v>42</v>
@@ -2166,7 +2163,7 @@
         <v>43</v>
       </c>
       <c r="N11" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>44</v>
@@ -2199,19 +2196,19 @@
         <v>50</v>
       </c>
       <c r="Y11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z11" t="s">
         <v>51</v>
       </c>
       <c r="AA11" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB11" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD11" t="s">
         <v>52</v>
@@ -2228,10 +2225,10 @@
         <v>38</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>39</v>
@@ -2252,7 +2249,7 @@
         <v>40</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>42</v>
@@ -2261,7 +2258,7 @@
         <v>43</v>
       </c>
       <c r="N12" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O12" s="3" t="s">
         <v>44</v>
@@ -2294,19 +2291,19 @@
         <v>50</v>
       </c>
       <c r="Y12" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z12" s="4" t="s">
         <v>51</v>
       </c>
       <c r="AA12" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB12" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD12" t="s">
         <v>52</v>
@@ -2323,10 +2320,10 @@
         <v>38</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>39</v>
@@ -2347,7 +2344,7 @@
         <v>40</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>42</v>
@@ -2356,7 +2353,7 @@
         <v>43</v>
       </c>
       <c r="N13" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="O13" s="3" t="s">
         <v>44</v>
@@ -2389,19 +2386,19 @@
         <v>50</v>
       </c>
       <c r="Y13" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z13" s="4" t="s">
         <v>51</v>
       </c>
       <c r="AA13" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AB13" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD13" t="s">
         <v>52</v>
@@ -2427,7 +2424,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2437,22 +2434,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -2545,30 +2542,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C2" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2576,16 +2573,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C3" t="s">
         <v>42</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -2593,16 +2590,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C4" t="s">
         <v>42</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -2610,16 +2607,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2627,16 +2624,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>42</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -2644,16 +2641,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C7" t="s">
         <v>42</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -2661,16 +2658,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E8">
         <v>7</v>
@@ -2678,16 +2675,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C9" t="s">
         <v>42</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E9">
         <v>8</v>
@@ -2695,16 +2692,16 @@
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -2712,16 +2709,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -2729,16 +2726,16 @@
     </row>
     <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E12">
         <v>11</v>
@@ -2746,10 +2743,10 @@
     </row>
     <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>42</v>
@@ -2773,267 +2770,267 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
locator changes May 13 24- 1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B80AA7-E63F-4277-90B1-5BE1C0EFE54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FA857C-EACC-49E5-98D9-46F52701595B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="171">
   <si>
     <t>James Craven</t>
   </si>
@@ -535,13 +535,37 @@
   </si>
   <si>
     <t>Business Services</t>
+  </si>
+  <si>
+    <t>Alex Herrera</t>
+  </si>
+  <si>
+    <t>Alex Shuleschenko</t>
+  </si>
+  <si>
+    <t>Alex St. Pierre</t>
+  </si>
+  <si>
+    <t>Alex Krakovsky</t>
+  </si>
+  <si>
+    <t>Alex Lerer</t>
+  </si>
+  <si>
+    <t>Alex Orlean</t>
+  </si>
+  <si>
+    <t>Alex Raskin</t>
+  </si>
+  <si>
+    <t>Alex Sullivan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -572,6 +596,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -651,7 +682,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -672,6 +703,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -954,14 +986,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -972,7 +1004,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -988,13 +1020,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72C63D9-9284-4C4B-9F1D-16D1550F550E}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>54</v>
       </c>
@@ -1002,12 +1034,12 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>157</v>
       </c>
@@ -1020,13 +1052,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938FB3C8-D05A-4A1D-9559-104A9F0AD28A}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="56.7109375" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="1" max="1" width="56.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>158</v>
       </c>
@@ -1034,7 +1066,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>160</v>
       </c>
@@ -1042,7 +1074,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>160</v>
       </c>
@@ -1058,13 +1090,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204DA895-5616-4092-9340-8DD85852997B}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1075,7 +1107,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1086,7 +1118,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1102,17 +1134,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1125,22 +1157,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -1154,28 +1186,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="29" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="5.28515625" customWidth="1"/>
+    <col min="26" max="26" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="5.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1267,7 +1299,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -1362,7 +1394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1457,7 +1489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -1552,7 +1584,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1647,7 +1679,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1742,7 +1774,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1837,7 +1869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1932,7 +1964,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -2027,7 +2059,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -2122,7 +2154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -2217,7 +2249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>38</v>
       </c>
@@ -2312,7 +2344,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>38</v>
       </c>
@@ -2417,37 +2449,37 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD3AFCB-FF3D-4430-A7EF-EB1CDD64D866}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>71</v>
       </c>
@@ -2460,19 +2492,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -2498,7 +2530,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -2532,15 +2564,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF5C07A2-98E8-49FB-8166-32C99B1B07D9}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>94</v>
       </c>
@@ -2554,7 +2586,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>98</v>
       </c>
@@ -2571,7 +2603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>98</v>
       </c>
@@ -2588,7 +2620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>98</v>
       </c>
@@ -2605,7 +2637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>98</v>
       </c>
@@ -2622,7 +2654,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>98</v>
       </c>
@@ -2639,7 +2671,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>98</v>
       </c>
@@ -2656,7 +2688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>98</v>
       </c>
@@ -2673,7 +2705,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>98</v>
       </c>
@@ -2690,7 +2722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>98</v>
       </c>
@@ -2707,7 +2739,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>98</v>
       </c>
@@ -2724,7 +2756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>98</v>
       </c>
@@ -2741,7 +2773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>98</v>
       </c>
@@ -2762,273 +2794,302 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AF4DCB0-85D6-4076-87FF-4126675E54C9}">
-  <dimension ref="A1:A53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>167</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>169</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>170</v>
+      </c>
+      <c r="B52" s="12" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>154</v>
       </c>

</xml_diff>

<commit_message>
Add Contact of Eng page may 15 -1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FA857C-EACC-49E5-98D9-46F52701595B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680D6EA8-847E-40C9-A0D8-AF1861CFB1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -986,14 +986,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -1020,13 +1020,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72C63D9-9284-4C4B-9F1D-16D1550F550E}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>54</v>
       </c>
@@ -1034,12 +1034,12 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>157</v>
       </c>
@@ -1052,13 +1052,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938FB3C8-D05A-4A1D-9559-104A9F0AD28A}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="56.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="1" max="1" width="56.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>158</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>160</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>160</v>
       </c>
@@ -1090,13 +1090,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204DA895-5616-4092-9340-8DD85852997B}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1134,17 +1134,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1157,22 +1157,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -1186,28 +1186,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="29" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="5.33203125" customWidth="1"/>
+    <col min="26" max="26" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="5.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1299,7 +1299,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -2154,7 +2154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>38</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>38</v>
       </c>
@@ -2449,37 +2449,37 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD3AFCB-FF3D-4430-A7EF-EB1CDD64D866}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>71</v>
       </c>
@@ -2492,19 +2492,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -2564,15 +2564,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF5C07A2-98E8-49FB-8166-32C99B1B07D9}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>94</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>98</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>98</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>98</v>
       </c>
@@ -2637,7 +2637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>98</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>98</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>98</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>98</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>98</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>98</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>98</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>98</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>98</v>
       </c>
@@ -2795,49 +2795,49 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AF4DCB0-85D6-4076-87FF-4126675E54C9}">
   <dimension ref="A1:D53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>163</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>110</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>111</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>166</v>
       </c>
@@ -2869,7 +2869,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>113</v>
       </c>
@@ -2877,62 +2877,62 @@
         <v>149</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>167</v>
       </c>
@@ -2940,67 +2940,67 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>168</v>
       </c>
@@ -3008,32 +3008,32 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>169</v>
       </c>
@@ -3041,47 +3041,47 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>170</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>154</v>
       </c>

</xml_diff>

<commit_message>
contactsname locator updated may 15 24 2
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680D6EA8-847E-40C9-A0D8-AF1861CFB1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE93584-8284-44DB-BEC3-63B192489DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="172">
   <si>
     <t>James Craven</t>
   </si>
@@ -559,6 +559,9 @@
   </si>
   <si>
     <t>Alex Sullivan</t>
+  </si>
+  <si>
+    <t>Chris1 Lord1</t>
   </si>
 </sst>
 </file>
@@ -2532,7 +2535,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
July 8 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738D4813-E2CA-4546-A84A-34E45D5F0976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7BDC43-AA60-414C-9256-091766D806F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="171">
   <si>
     <t>James Craven</t>
   </si>
@@ -553,9 +553,6 @@
   </si>
   <si>
     <t>Alex Sullivan</t>
-  </si>
-  <si>
-    <t>Chris1 Lord1</t>
   </si>
   <si>
     <t>CSDN-0000007327</t>
@@ -1221,7 +1218,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1313,7 +1310,7 @@
         <v>73</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
@@ -1408,7 +1405,7 @@
         <v>81</v>
       </c>
       <c r="D3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
@@ -1503,7 +1500,7 @@
         <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E4" t="s">
         <v>38</v>
@@ -1598,7 +1595,7 @@
         <v>83</v>
       </c>
       <c r="D5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -1693,7 +1690,7 @@
         <v>84</v>
       </c>
       <c r="D6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
@@ -1788,7 +1785,7 @@
         <v>85</v>
       </c>
       <c r="D7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E7" t="s">
         <v>38</v>
@@ -1883,7 +1880,7 @@
         <v>86</v>
       </c>
       <c r="D8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
@@ -1978,7 +1975,7 @@
         <v>87</v>
       </c>
       <c r="D9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -2073,7 +2070,7 @@
         <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E10" t="s">
         <v>38</v>
@@ -2168,7 +2165,7 @@
         <v>89</v>
       </c>
       <c r="D11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E11" t="s">
         <v>38</v>
@@ -2263,7 +2260,7 @@
         <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>38</v>
@@ -2358,7 +2355,7 @@
         <v>91</v>
       </c>
       <c r="D13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>38</v>
@@ -2535,7 +2532,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>169</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
CAO Users  updated May 16 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D72455C-5700-4801-A556-1F6AD0607050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638087AE-E166-4023-B63C-10184959F379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -283,9 +283,6 @@
     <t>10000</t>
   </si>
   <si>
-    <t>Liz Hedgcock</t>
-  </si>
-  <si>
     <t>Tombstone Permission</t>
   </si>
   <si>
@@ -566,6 +563,9 @@
   </si>
   <si>
     <t>Legal Hold test Notes</t>
+  </si>
+  <si>
+    <t>Blaise Brunda</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1013,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1038,17 +1038,17 @@
         <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -1067,26 +1067,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1104,12 +1104,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -1139,7 +1139,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>172</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1153,23 +1153,23 @@
         <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" t="s">
         <v>169</v>
-      </c>
-      <c r="B5" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1264,7 +1264,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1339,7 +1339,7 @@
         <v>35</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>36</v>
@@ -1356,7 +1356,7 @@
         <v>73</v>
       </c>
       <c r="D2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
@@ -1386,7 +1386,7 @@
         <v>42</v>
       </c>
       <c r="N2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>43</v>
@@ -1431,7 +1431,7 @@
         <v>77</v>
       </c>
       <c r="AC2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD2" t="s">
         <v>51</v>
@@ -1448,10 +1448,10 @@
         <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
@@ -1481,7 +1481,7 @@
         <v>42</v>
       </c>
       <c r="N3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>43</v>
@@ -1526,7 +1526,7 @@
         <v>77</v>
       </c>
       <c r="AC3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD3" t="s">
         <v>39</v>
@@ -1543,10 +1543,10 @@
         <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E4" t="s">
         <v>38</v>
@@ -1576,7 +1576,7 @@
         <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>43</v>
@@ -1621,7 +1621,7 @@
         <v>77</v>
       </c>
       <c r="AC4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD4" t="s">
         <v>51</v>
@@ -1638,10 +1638,10 @@
         <v>37</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -1671,7 +1671,7 @@
         <v>42</v>
       </c>
       <c r="N5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>43</v>
@@ -1716,7 +1716,7 @@
         <v>77</v>
       </c>
       <c r="AC5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD5" t="s">
         <v>39</v>
@@ -1733,10 +1733,10 @@
         <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
@@ -1766,7 +1766,7 @@
         <v>42</v>
       </c>
       <c r="N6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>43</v>
@@ -1811,7 +1811,7 @@
         <v>77</v>
       </c>
       <c r="AC6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD6" t="s">
         <v>51</v>
@@ -1828,10 +1828,10 @@
         <v>37</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E7" t="s">
         <v>38</v>
@@ -1861,7 +1861,7 @@
         <v>42</v>
       </c>
       <c r="N7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>43</v>
@@ -1906,7 +1906,7 @@
         <v>77</v>
       </c>
       <c r="AC7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD7" t="s">
         <v>39</v>
@@ -1923,10 +1923,10 @@
         <v>37</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
@@ -1956,7 +1956,7 @@
         <v>42</v>
       </c>
       <c r="N8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>43</v>
@@ -2001,7 +2001,7 @@
         <v>77</v>
       </c>
       <c r="AC8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD8" t="s">
         <v>51</v>
@@ -2018,10 +2018,10 @@
         <v>37</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -2051,7 +2051,7 @@
         <v>42</v>
       </c>
       <c r="N9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>43</v>
@@ -2096,7 +2096,7 @@
         <v>77</v>
       </c>
       <c r="AC9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD9" t="s">
         <v>39</v>
@@ -2113,10 +2113,10 @@
         <v>37</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E10" t="s">
         <v>38</v>
@@ -2146,7 +2146,7 @@
         <v>42</v>
       </c>
       <c r="N10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>43</v>
@@ -2191,7 +2191,7 @@
         <v>77</v>
       </c>
       <c r="AC10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD10" t="s">
         <v>51</v>
@@ -2208,10 +2208,10 @@
         <v>37</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E11" t="s">
         <v>38</v>
@@ -2241,7 +2241,7 @@
         <v>42</v>
       </c>
       <c r="N11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>43</v>
@@ -2286,7 +2286,7 @@
         <v>77</v>
       </c>
       <c r="AC11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AD11" t="s">
         <v>51</v>
@@ -2430,24 +2430,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C2" t="s">
         <v>41</v>
@@ -2461,16 +2461,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C3" t="s">
         <v>41</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -2478,16 +2478,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C4" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -2495,16 +2495,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C5" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2512,16 +2512,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -2529,16 +2529,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C7" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -2546,16 +2546,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C8" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E8">
         <v>7</v>
@@ -2563,16 +2563,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E9">
         <v>8</v>
@@ -2580,16 +2580,16 @@
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -2597,16 +2597,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -2629,294 +2629,294 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
may 16 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
+++ b/TestData/LV_T1432_OpportunityToEngagementConversionMappingForFVAJobTypes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638087AE-E166-4023-B63C-10184959F379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{754AEB46-C973-49AE-9335-A12E3428CBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -265,9 +265,6 @@
     <t>Engagements</t>
   </si>
   <si>
-    <t>Indrajeet Singh</t>
-  </si>
-  <si>
     <t>FA - Portfolio-Advis/Consulting</t>
   </si>
   <si>
@@ -566,6 +563,9 @@
   </si>
   <si>
     <t>Blaise Brunda</t>
+  </si>
+  <si>
+    <t>Ajay Nair</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1013,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1038,17 +1038,17 @@
         <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1067,26 +1067,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1104,12 +1104,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1139,7 +1139,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1150,26 +1150,26 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>172</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" t="s">
         <v>166</v>
-      </c>
-      <c r="B4" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" t="s">
         <v>168</v>
-      </c>
-      <c r="B5" t="s">
-        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1264,7 +1264,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1330,7 +1330,7 @@
         <v>33</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>34</v>
@@ -1339,7 +1339,7 @@
         <v>35</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>36</v>
@@ -1353,10 +1353,10 @@
         <v>37</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
@@ -1377,7 +1377,7 @@
         <v>39</v>
       </c>
       <c r="K2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L2" t="s">
         <v>41</v>
@@ -1386,7 +1386,7 @@
         <v>42</v>
       </c>
       <c r="N2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>43</v>
@@ -1419,19 +1419,19 @@
         <v>49</v>
       </c>
       <c r="Y2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z2" t="s">
         <v>50</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD2" t="s">
         <v>51</v>
@@ -1448,10 +1448,10 @@
         <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
@@ -1472,7 +1472,7 @@
         <v>39</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L3" t="s">
         <v>41</v>
@@ -1481,7 +1481,7 @@
         <v>42</v>
       </c>
       <c r="N3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>43</v>
@@ -1514,19 +1514,19 @@
         <v>49</v>
       </c>
       <c r="Y3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z3" t="s">
         <v>50</v>
       </c>
       <c r="AA3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD3" t="s">
         <v>39</v>
@@ -1543,10 +1543,10 @@
         <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E4" t="s">
         <v>38</v>
@@ -1567,7 +1567,7 @@
         <v>39</v>
       </c>
       <c r="K4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L4" t="s">
         <v>41</v>
@@ -1576,7 +1576,7 @@
         <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>43</v>
@@ -1609,19 +1609,19 @@
         <v>49</v>
       </c>
       <c r="Y4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z4" t="s">
         <v>50</v>
       </c>
       <c r="AA4" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB4" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD4" t="s">
         <v>51</v>
@@ -1638,10 +1638,10 @@
         <v>37</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -1662,7 +1662,7 @@
         <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L5" t="s">
         <v>41</v>
@@ -1671,7 +1671,7 @@
         <v>42</v>
       </c>
       <c r="N5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>43</v>
@@ -1704,19 +1704,19 @@
         <v>49</v>
       </c>
       <c r="Y5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z5" t="s">
         <v>50</v>
       </c>
       <c r="AA5" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD5" t="s">
         <v>39</v>
@@ -1733,10 +1733,10 @@
         <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
@@ -1757,7 +1757,7 @@
         <v>39</v>
       </c>
       <c r="K6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L6" t="s">
         <v>41</v>
@@ -1766,7 +1766,7 @@
         <v>42</v>
       </c>
       <c r="N6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>43</v>
@@ -1799,19 +1799,19 @@
         <v>49</v>
       </c>
       <c r="Y6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z6" t="s">
         <v>50</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB6" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD6" t="s">
         <v>51</v>
@@ -1828,10 +1828,10 @@
         <v>37</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E7" t="s">
         <v>38</v>
@@ -1852,7 +1852,7 @@
         <v>39</v>
       </c>
       <c r="K7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L7" t="s">
         <v>41</v>
@@ -1861,7 +1861,7 @@
         <v>42</v>
       </c>
       <c r="N7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>43</v>
@@ -1894,19 +1894,19 @@
         <v>49</v>
       </c>
       <c r="Y7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z7" t="s">
         <v>50</v>
       </c>
       <c r="AA7" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD7" t="s">
         <v>39</v>
@@ -1923,10 +1923,10 @@
         <v>37</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
@@ -1947,7 +1947,7 @@
         <v>39</v>
       </c>
       <c r="K8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L8" t="s">
         <v>41</v>
@@ -1956,7 +1956,7 @@
         <v>42</v>
       </c>
       <c r="N8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>43</v>
@@ -1989,19 +1989,19 @@
         <v>49</v>
       </c>
       <c r="Y8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z8" t="s">
         <v>50</v>
       </c>
       <c r="AA8" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB8" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD8" t="s">
         <v>51</v>
@@ -2018,10 +2018,10 @@
         <v>37</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -2042,7 +2042,7 @@
         <v>39</v>
       </c>
       <c r="K9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L9" t="s">
         <v>41</v>
@@ -2051,7 +2051,7 @@
         <v>42</v>
       </c>
       <c r="N9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>43</v>
@@ -2084,19 +2084,19 @@
         <v>49</v>
       </c>
       <c r="Y9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z9" t="s">
         <v>50</v>
       </c>
       <c r="AA9" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB9" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD9" t="s">
         <v>39</v>
@@ -2113,10 +2113,10 @@
         <v>37</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E10" t="s">
         <v>38</v>
@@ -2137,7 +2137,7 @@
         <v>39</v>
       </c>
       <c r="K10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L10" t="s">
         <v>41</v>
@@ -2146,7 +2146,7 @@
         <v>42</v>
       </c>
       <c r="N10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>43</v>
@@ -2179,19 +2179,19 @@
         <v>49</v>
       </c>
       <c r="Y10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z10" t="s">
         <v>50</v>
       </c>
       <c r="AA10" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB10" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD10" t="s">
         <v>51</v>
@@ -2208,10 +2208,10 @@
         <v>37</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E11" t="s">
         <v>38</v>
@@ -2232,7 +2232,7 @@
         <v>39</v>
       </c>
       <c r="K11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L11" t="s">
         <v>41</v>
@@ -2241,7 +2241,7 @@
         <v>42</v>
       </c>
       <c r="N11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>43</v>
@@ -2274,19 +2274,19 @@
         <v>49</v>
       </c>
       <c r="Y11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z11" t="s">
         <v>50</v>
       </c>
       <c r="AA11" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB11" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AC11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AD11" t="s">
         <v>51</v>
@@ -2430,30 +2430,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C2" t="s">
         <v>41</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2461,16 +2461,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C3" t="s">
         <v>41</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -2478,16 +2478,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C4" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -2495,16 +2495,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C5" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2512,16 +2512,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -2529,16 +2529,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C7" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -2546,16 +2546,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C8" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E8">
         <v>7</v>
@@ -2563,16 +2563,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E9">
         <v>8</v>
@@ -2580,16 +2580,16 @@
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -2597,16 +2597,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>95</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -2629,294 +2629,294 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>